<commit_message>
Add portal checklist tab to the client getting-started workbook
</commit_message>
<xml_diff>
--- a/docs/client-forms/Kingaroy-portal-getting-started.xlsx
+++ b/docs/client-forms/Kingaroy-portal-getting-started.xlsx
@@ -8,12 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production steps" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order cycles" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portal checklist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production steps" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order cycles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payments" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Portal checklist'!$4:$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,8 +87,26 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color theme="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -107,8 +128,13 @@
         <fgColor rgb="00FFF7D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1E8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -130,11 +156,12 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -168,6 +195,27 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -535,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -571,7 +619,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>• Grey rows are examples only, to show the format. Please leave them or type over them.</t>
+          <t>• Grey cells are examples only, to show the format. Please leave them or type over them.</t>
         </is>
       </c>
     </row>
@@ -600,45 +648,52 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>1. Suppliers: who you buy garments from. Only the supplier name is essential; the rest is optional.</t>
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>1. Portal checklist: how each customer's portal should work (budgets, approvals, payments and so on). One column per customer.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2. Production steps: what happens to an order from the moment it arrives until it's dispatched.</t>
+          <t>2. Suppliers: who you buy garments from. Only the supplier name is essential; the rest is optional.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>3. Order cycles: whether you pool orders and send them to production on set days.</t>
+          <t>3. Production steps: what happens to an order from the moment it arrives until it's dispatched.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>4. Payments: how you take card payments today.</t>
+          <t>4. Order cycles: whether you pool orders and send them to production on set days.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>5. Payments: how you take card payments today.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Separately, a customer export from Xero (business name only is fine) covers who you supply.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Please don't put passwords, card numbers or login details anywhere in this workbook.</t>
         </is>
@@ -650,6 +705,1258 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Portal checklist</t>
+        </is>
+      </c>
+      <c r="J1" s="23" t="n"/>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>One column per customer portal. Put the customer's name in the top yellow cell, then pick an answer from the drop-down in each row (or type your own). Amounts, names and anything unusual go in Notes. The grey column is an example only. Not sure? Leave it blank, and we'll go through it together.</t>
+        </is>
+      </c>
+      <c r="J2" s="23" t="n"/>
+    </row>
+    <row r="3">
+      <c r="J3" s="23" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Choices</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Portal 1</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Portal 2</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Portal 3</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Portal 4</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>Portal 5</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Customer / portal name</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n"/>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Example Childcare Centre</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="24" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Setup and access</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n"/>
+      <c r="C6" s="20" t="n"/>
+      <c r="D6" s="20" t="n"/>
+      <c r="E6" s="20" t="n"/>
+      <c r="F6" s="20" t="n"/>
+      <c r="G6" s="20" t="n"/>
+      <c r="H6" s="20" t="n"/>
+      <c r="I6" s="20" t="n"/>
+      <c r="J6" s="23" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>How is the portal set up?</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>One portal for the whole organisation · One portal per centre · Group portal with centres inside</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Group portal with centres inside</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="11" t="n"/>
+      <c r="I7" s="11" t="n"/>
+      <c r="J7" s="25" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>How will staff get an account?</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>We upload a staff list · Staff sign up themselves · Sign-up limited to work email</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Staff sign up themselves</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="11" t="n"/>
+      <c r="I8" s="11" t="n"/>
+      <c r="J8" s="25" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Do new sign-ups need approving?</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>No · Yes - centre manager · Yes - organisation admin</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Yes - centre manager</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
+      <c r="I9" s="11" t="n"/>
+      <c r="J9" s="25" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Who removes staff who leave?</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>Centre manager · Organisation admin · Kingaroy</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Centre manager</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="11" t="n"/>
+      <c r="I10" s="11" t="n"/>
+      <c r="J10" s="25" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>What happens to a leaver's unused budget?</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>Lost · Returned to the centre · No budgets</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Lost</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="11" t="n"/>
+      <c r="J11" s="25" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>A director-only page for bulk centre orders?</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="11" t="n"/>
+      <c r="I12" s="11" t="n"/>
+      <c r="J12" s="25" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>Any products or prices only directors should see? (list in notes)</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="11" t="n"/>
+      <c r="I13" s="11" t="n"/>
+      <c r="J13" s="25" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>Budgets</t>
+        </is>
+      </c>
+      <c r="B14" s="20" t="n"/>
+      <c r="C14" s="20" t="n"/>
+      <c r="D14" s="20" t="n"/>
+      <c r="E14" s="20" t="n"/>
+      <c r="F14" s="20" t="n"/>
+      <c r="G14" s="20" t="n"/>
+      <c r="H14" s="20" t="n"/>
+      <c r="I14" s="20" t="n"/>
+      <c r="J14" s="23" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>A budget per staff member? (amount in notes)</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="11" t="n"/>
+      <c r="I15" s="11" t="n"/>
+      <c r="J15" s="25" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>A budget per centre? (amount in notes)</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="11" t="n"/>
+      <c r="I16" s="11" t="n"/>
+      <c r="J16" s="25" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Budget period</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>Financial year · Calendar year · From each person's start date · Custom dates</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Financial year</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="11" t="n"/>
+      <c r="I17" s="11" t="n"/>
+      <c r="J17" s="25" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>At the end of the period</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>Resets · Unused balance rolls over</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Resets</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="11" t="n"/>
+      <c r="I18" s="11" t="n"/>
+      <c r="J18" s="25" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>New starters get</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>Full allowance straight away · Part now and the rest later</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Part now and the rest later</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
+      <c r="H19" s="11" t="n"/>
+      <c r="I19" s="11" t="n"/>
+      <c r="J19" s="25" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>Budgets are released</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>All at once · Centre by centre through the year</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>All at once</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
+      <c r="H20" s="11" t="n"/>
+      <c r="I20" s="11" t="n"/>
+      <c r="J20" s="25" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>The budget covers</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>Garments only · Garments and logo · Garments and logo and freight</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Garments and logo</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="11" t="n"/>
+      <c r="H21" s="11" t="n"/>
+      <c r="I21" s="11" t="n"/>
+      <c r="J21" s="25" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Separate budgets for garments and for logos?</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="11" t="n"/>
+      <c r="H22" s="11" t="n"/>
+      <c r="I22" s="11" t="n"/>
+      <c r="J22" s="25" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>When the budget runs out</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Block the order · Pay the difference by card · Send for approval</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Pay the difference by card</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+      <c r="G23" s="11" t="n"/>
+      <c r="H23" s="11" t="n"/>
+      <c r="I23" s="11" t="n"/>
+      <c r="J23" s="25" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Reminder emails before a budget expires?</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
+      <c r="G24" s="11" t="n"/>
+      <c r="H24" s="11" t="n"/>
+      <c r="I24" s="11" t="n"/>
+      <c r="J24" s="25" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Approvals and limits</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="20" t="n"/>
+      <c r="E25" s="20" t="n"/>
+      <c r="F25" s="20" t="n"/>
+      <c r="G25" s="20" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="20" t="n"/>
+      <c r="J25" s="23" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Do orders need approving?</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>No · All orders · Orders over an amount · Orders over budget · Certain products only</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Orders over budget</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="11" t="n"/>
+      <c r="G26" s="11" t="n"/>
+      <c r="H26" s="11" t="n"/>
+      <c r="I26" s="11" t="n"/>
+      <c r="J26" s="25" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t>Who approves orders?</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>Director · Organisation admin · Named person (in notes) · No approvals</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="11" t="n"/>
+      <c r="H27" s="11" t="n"/>
+      <c r="I27" s="11" t="n"/>
+      <c r="J27" s="25" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Minimum order?</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>None · Minimum dollar value · Minimum quantity</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="11" t="n"/>
+      <c r="H28" s="11" t="n"/>
+      <c r="I28" s="11" t="n"/>
+      <c r="J28" s="25" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>Maximum order?</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>None · Maximum per order · Maximum of an item per person per year</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Maximum of an item per person per year</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="11" t="n"/>
+      <c r="H29" s="11" t="n"/>
+      <c r="I29" s="11" t="n"/>
+      <c r="J29" s="25" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n"/>
+      <c r="C30" s="20" t="n"/>
+      <c r="D30" s="20" t="n"/>
+      <c r="E30" s="20" t="n"/>
+      <c r="F30" s="20" t="n"/>
+      <c r="G30" s="20" t="n"/>
+      <c r="H30" s="20" t="n"/>
+      <c r="I30" s="20" t="n"/>
+      <c r="J30" s="23" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>Can staff buy extra uniform at their own cost?</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="11" t="n"/>
+      <c r="I31" s="11" t="n"/>
+      <c r="J31" s="25" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>Different prices for staff purchases and centre orders?</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="11" t="n"/>
+      <c r="H32" s="11" t="n"/>
+      <c r="I32" s="11" t="n"/>
+      <c r="J32" s="25" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>Centre and bulk orders are paid by</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>On account (invoice) · Card · Either</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>On account (invoice)</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="11" t="n"/>
+      <c r="H33" s="11" t="n"/>
+      <c r="I33" s="11" t="n"/>
+      <c r="J33" s="25" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>Card surcharge?</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="11" t="n"/>
+      <c r="F34" s="11" t="n"/>
+      <c r="G34" s="11" t="n"/>
+      <c r="H34" s="11" t="n"/>
+      <c r="I34" s="11" t="n"/>
+      <c r="J34" s="25" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>Where should invoices and order copies go? (a work inbox such as accounts@)</t>
+        </is>
+      </c>
+      <c r="B35" s="22" t="inlineStr">
+        <is>
+          <t>Type the answer</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>accounts@ inbox</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="n"/>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="11" t="n"/>
+      <c r="G35" s="11" t="n"/>
+      <c r="H35" s="11" t="n"/>
+      <c r="I35" s="11" t="n"/>
+      <c r="J35" s="25" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>Freight and delivery</t>
+        </is>
+      </c>
+      <c r="B36" s="20" t="n"/>
+      <c r="C36" s="20" t="n"/>
+      <c r="D36" s="20" t="n"/>
+      <c r="E36" s="20" t="n"/>
+      <c r="F36" s="20" t="n"/>
+      <c r="G36" s="20" t="n"/>
+      <c r="H36" s="20" t="n"/>
+      <c r="I36" s="20" t="n"/>
+      <c r="J36" s="23" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>Freight</t>
+        </is>
+      </c>
+      <c r="B37" s="22" t="inlineStr">
+        <is>
+          <t>Free · Flat rate · Free over an amount · Free whenever a budget is used</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>Free whenever a budget is used</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="11" t="n"/>
+      <c r="H37" s="11" t="n"/>
+      <c r="I37" s="11" t="n"/>
+      <c r="J37" s="25" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>Deliver to</t>
+        </is>
+      </c>
+      <c r="B38" s="22" t="inlineStr">
+        <is>
+          <t>Centre only · Centre or home address</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>Centre only</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="11" t="n"/>
+      <c r="G38" s="11" t="n"/>
+      <c r="H38" s="11" t="n"/>
+      <c r="I38" s="11" t="n"/>
+      <c r="J38" s="25" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>Orders go to production</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>As they come in · On set days with a cut-off</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>On set days with a cut-off</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="11" t="n"/>
+      <c r="H39" s="11" t="n"/>
+      <c r="I39" s="11" t="n"/>
+      <c r="J39" s="25" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>Products, logos and sizing</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="n"/>
+      <c r="C40" s="20" t="n"/>
+      <c r="D40" s="20" t="n"/>
+      <c r="E40" s="20" t="n"/>
+      <c r="F40" s="20" t="n"/>
+      <c r="G40" s="20" t="n"/>
+      <c r="H40" s="20" t="n"/>
+      <c r="I40" s="20" t="n"/>
+      <c r="J40" s="23" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>Logos</t>
+        </is>
+      </c>
+      <c r="B41" s="22" t="inlineStr">
+        <is>
+          <t>One logo on everything · A logo per centre · Group logo and centre logo</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>One logo on everything</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="11" t="n"/>
+      <c r="H41" s="11" t="n"/>
+      <c r="I41" s="11" t="n"/>
+      <c r="J41" s="25" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>Logo setup fee</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>We absorb it · Charged to the customer · Built into prices</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>Built into prices</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="11" t="n"/>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="11" t="n"/>
+      <c r="H42" s="11" t="n"/>
+      <c r="I42" s="11" t="n"/>
+      <c r="J42" s="25" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>Names or roles embroidered on garments?</t>
+        </is>
+      </c>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="11" t="n"/>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11" t="n"/>
+      <c r="H43" s="11" t="n"/>
+      <c r="I43" s="11" t="n"/>
+      <c r="J43" s="25" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>Starter packs for new staff?</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="n"/>
+      <c r="E44" s="11" t="n"/>
+      <c r="F44" s="11" t="n"/>
+      <c r="G44" s="11" t="n"/>
+      <c r="H44" s="11" t="n"/>
+      <c r="I44" s="11" t="n"/>
+      <c r="J44" s="25" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="21" t="inlineStr">
+        <is>
+          <t>Size registration before ordering (e.g. a fitting day)?</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="n"/>
+      <c r="E45" s="11" t="n"/>
+      <c r="F45" s="11" t="n"/>
+      <c r="G45" s="11" t="n"/>
+      <c r="H45" s="11" t="n"/>
+      <c r="I45" s="11" t="n"/>
+      <c r="J45" s="25" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="21" t="inlineStr">
+        <is>
+          <t>Easy wrong-size swaps?</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="11" t="n"/>
+      <c r="F46" s="11" t="n"/>
+      <c r="G46" s="11" t="n"/>
+      <c r="H46" s="11" t="n"/>
+      <c r="I46" s="11" t="n"/>
+      <c r="J46" s="25" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t>Look and messages</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="n"/>
+      <c r="C47" s="20" t="n"/>
+      <c r="D47" s="20" t="n"/>
+      <c r="E47" s="20" t="n"/>
+      <c r="F47" s="20" t="n"/>
+      <c r="G47" s="20" t="n"/>
+      <c r="H47" s="20" t="n"/>
+      <c r="I47" s="20" t="n"/>
+      <c r="J47" s="23" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="21" t="inlineStr">
+        <is>
+          <t>Branding (logo, colours, welcome text)</t>
+        </is>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>Customer supplies it · Kingaroy designs it</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>Customer supplies it</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="11" t="n"/>
+      <c r="F48" s="11" t="n"/>
+      <c r="G48" s="11" t="n"/>
+      <c r="H48" s="11" t="n"/>
+      <c r="I48" s="11" t="n"/>
+      <c r="J48" s="25" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="21" t="inlineStr">
+        <is>
+          <t>Portal web address</t>
+        </is>
+      </c>
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>Customer's own address · Address provided by Kingaroy</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>Address provided by Kingaroy</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="n"/>
+      <c r="E49" s="11" t="n"/>
+      <c r="F49" s="11" t="n"/>
+      <c r="G49" s="11" t="n"/>
+      <c r="H49" s="11" t="n"/>
+      <c r="I49" s="11" t="n"/>
+      <c r="J49" s="25" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>Store notices (e.g. holiday closures)?</t>
+        </is>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>Yes · No</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="11" t="n"/>
+      <c r="F50" s="11" t="n"/>
+      <c r="G50" s="11" t="n"/>
+      <c r="H50" s="11" t="n"/>
+      <c r="I50" s="11" t="n"/>
+      <c r="J50" s="25" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <dataValidations count="37">
+    <dataValidation sqref="D7:H7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"One portal for the whole organisation,One portal per centre,Group portal with centres inside"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D8:H8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"We upload a staff list,Staff sign up themselves,Sign-up limited to work email"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D9:H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No,Yes - centre manager,Yes - organisation admin"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D10:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Centre manager,Organisation admin,Kingaroy"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D11:H11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Lost,Returned to the centre,No budgets"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D12:H12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D13:H13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D15:H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D16:H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D17:H17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Financial year,Calendar year,From each person's start date,Custom dates"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D18:H18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Resets,Unused balance rolls over"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D19:H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Full allowance straight away,Part now and the rest later"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D20:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"All at once,Centre by centre through the year"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D21:H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Garments only,Garments and logo,Garments and logo and freight"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D22:H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D23:H23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Block the order,Pay the difference by card,Send for approval"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D24:H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D26:H26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"No,All orders,Orders over an amount,Orders over budget,Certain products only"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D27:H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Director,Organisation admin,Named person (in notes),No approvals"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D28:H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"None,Minimum dollar value,Minimum quantity"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D29:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"None,Maximum per order,Maximum of an item per person per year"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D31:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D32:H32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D33:H33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"On account (invoice),Card,Either"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D34:H34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D37:H37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Free,Flat rate,Free over an amount,Free whenever a budget is used"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D38:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Centre only,Centre or home address"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D39:H39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"As they come in,On set days with a cut-off"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D41:H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"One logo on everything,A logo per centre,Group logo and centre logo"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D42:H42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"We absorb it,Charged to the customer,Built into prices"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D43:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D44:H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D45:H45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D46:H46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D48:H48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Customer supplies it,Kingaroy designs it"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D49:H49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Customer's own address,Address provided by Kingaroy"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D50:H50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -872,7 +2179,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1069,7 +2376,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1288,7 +2595,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>